<commit_message>
Fix import infrastructure, title block model, and content structure
- Fix import path generation to use flat file structure (no folder/index pattern)
- Fix carousel parser to preserve lazy-loaded images from noscript tags
- Fix table parser with proper 6-column alignment and p-wrapped cells
- Remove tournament table from homepage import (md2jcr unsupported element)
- Update title block to use multiselect classes field for position and colour
- Add explicit left/center/right position and black/white/blue colour CSS classes
- Update cleanup transformer to strip tournament table section

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="41">
   <si>
     <t>_reportFile</t>
   </si>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-03-27T01:06:18.069Z</t>
+    <t>2026-04-02T01:05:49.367Z</t>
   </si>
   <si>
     <t>Tennis NSW | The governing body of Tennis in New South Wales</t>
@@ -61,6 +61,42 @@
     <t>https://www.tennis.com.au/nsw/</t>
   </si>
   <si>
+    <t>nsw/about-us.report.json</t>
+  </si>
+  <si>
+    <t>["cards"]</t>
+  </si>
+  <si>
+    <t>nsw/about-us</t>
+  </si>
+  <si>
+    <t>section-landing</t>
+  </si>
+  <si>
+    <t>2026-04-01T08:01:59.224Z</t>
+  </si>
+  <si>
+    <t>About Us | Tennis NSW</t>
+  </si>
+  <si>
+    <t>https://www.tennis.com.au/nsw/about-us</t>
+  </si>
+  <si>
+    <t>nsw/clubs.report.json</t>
+  </si>
+  <si>
+    <t>nsw/clubs</t>
+  </si>
+  <si>
+    <t>2026-04-01T08:01:43.787Z</t>
+  </si>
+  <si>
+    <t>Clubs | Tennis NSW</t>
+  </si>
+  <si>
+    <t>https://www.tennis.com.au/nsw/clubs</t>
+  </si>
+  <si>
     <t>nsw/index.report.json</t>
   </si>
   <si>
@@ -68,6 +104,36 @@
   </si>
   <si>
     <t>2026-03-27T01:07:17.044Z</t>
+  </si>
+  <si>
+    <t>nsw/our-work.report.json</t>
+  </si>
+  <si>
+    <t>nsw/our-work</t>
+  </si>
+  <si>
+    <t>2026-04-01T08:01:53.285Z</t>
+  </si>
+  <si>
+    <t>Our Work | Tennis NSW</t>
+  </si>
+  <si>
+    <t>https://www.tennis.com.au/nsw/our-work</t>
+  </si>
+  <si>
+    <t>nsw/players.report.json</t>
+  </si>
+  <si>
+    <t>nsw/players</t>
+  </si>
+  <si>
+    <t>2026-04-01T08:01:47.511Z</t>
+  </si>
+  <si>
+    <t>Play | Tennis NSW</t>
+  </si>
+  <si>
+    <t>https://www.tennis.com.au/nsw/players</t>
   </si>
 </sst>
 </file>
@@ -456,16 +522,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="23" customWidth="1"/>
+    <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="11" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="5" max="5" width="17" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="50" customWidth="1"/>
-    <col min="8" max="8" width="32" customWidth="1"/>
+    <col min="8" max="8" width="40" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -525,25 +591,129 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D3" t="s">
         <v>11</v>
       </c>
       <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
         <v>12</v>
       </c>
-      <c r="F3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="F5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" t="s">
         <v>14</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H5" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" t="s">
+        <v>38</v>
+      </c>
+      <c r="G7" t="s">
+        <v>39</v>
+      </c>
+      <c r="H7" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Extend card model to 4 fields: title, image, text, link
Card model now has separate fields for:
- title: plain text heading (displayed above image)
- image: card image reference
- text: richtext description
- link: CTA link URL with display text

Cards JS builds DOM as: heading → image → body → CTA link
matching original Tennis NSW card element order.

Parser outputs 4-cell rows. All 5 pages re-imported with fixes:
- Duplicate banners removed
- Title blocks, section metadata re-applied

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-04-02T06:11:05.694Z</t>
+    <t>2026-04-02T07:40:19.934Z</t>
   </si>
   <si>
     <t>Tennis NSW | The governing body of Tennis in New South Wales</t>
@@ -73,7 +73,7 @@
     <t>section-landing</t>
   </si>
   <si>
-    <t>2026-04-01T08:01:59.224Z</t>
+    <t>2026-04-02T07:13:02.390Z</t>
   </si>
   <si>
     <t>About Us | Tennis NSW</t>
@@ -88,7 +88,7 @@
     <t>nsw/clubs</t>
   </si>
   <si>
-    <t>2026-04-01T08:01:43.787Z</t>
+    <t>2026-04-02T07:29:12.200Z</t>
   </si>
   <si>
     <t>Clubs | Tennis NSW</t>
@@ -112,7 +112,7 @@
     <t>nsw/our-work</t>
   </si>
   <si>
-    <t>2026-04-01T08:01:53.285Z</t>
+    <t>2026-04-02T07:29:17.215Z</t>
   </si>
   <si>
     <t>Our Work | Tennis NSW</t>
@@ -127,7 +127,7 @@
     <t>nsw/players</t>
   </si>
   <si>
-    <t>2026-04-01T08:01:47.511Z</t>
+    <t>2026-04-02T07:12:57.410Z</t>
   </si>
   <si>
     <t>Play | Tennis NSW</t>

</xml_diff>